<commit_message>
client application added, dockerfile split and compose with a better structure
</commit_message>
<xml_diff>
--- a/Template_ATDD_Gamificacao.xlsx
+++ b/Template_ATDD_Gamificacao.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0748a122137392b1/Documentos/DevOps/pratica5/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Giovanne\Documents\DevOps\Pratica5-DevOps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="83" documentId="8_{0394F7CC-9F61-4387-A1CE-9B2407917102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1473AAC4-7B12-4970-BF2C-176E5A9E1C48}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F50062C5-1673-4CFF-BC08-08C09787F9C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pb" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="62">
   <si>
     <t>PRODUCT BACKLOG</t>
   </si>
@@ -417,58 +417,52 @@
     </r>
   </si>
   <si>
-    <t>Dado um aluno matriculado na plataforma</t>
-  </si>
-  <si>
-    <t>E com acesso liberado ao fórum de discussões</t>
-  </si>
-  <si>
-    <t>Quando o aluno publica um novo tópico</t>
-  </si>
-  <si>
-    <t>E outro participante comenta ajudando com uma resposta</t>
-  </si>
-  <si>
-    <t>Então as interações de ambos devem ser registradas</t>
-  </si>
-  <si>
-    <t>E as métricas de engajamento mensal de cada um devem ser incrementadas</t>
-  </si>
-  <si>
-    <t>Dado um aluno com 11 cursos concluídos com sucesso</t>
-  </si>
-  <si>
-    <t>E com plano de assinatura "Básica"</t>
-  </si>
-  <si>
-    <t>Quando ele conclui o seu 12º curso com nota maior ou igual a 8</t>
-  </si>
-  <si>
-    <t>E a conclusão é validada pelo sistema</t>
-  </si>
-  <si>
-    <t>Então o plano deve ser atualizado para "Premium"</t>
-  </si>
-  <si>
-    <t>E ele deve receber 3 novos cursos, 3 moedas e voucher para projetos reais</t>
-  </si>
-  <si>
-    <t>Dado um aluno Premium que liderou o ranking do fórum no mês</t>
-  </si>
-  <si>
-    <t>E possui saldo de 3 moedas acumuladas</t>
-  </si>
-  <si>
-    <t>Quando for processada a apuração mensal de gamificação</t>
-  </si>
-  <si>
-    <t>E o aluno solicitar a conversão de 1 moeda em criptomoeda</t>
-  </si>
-  <si>
-    <t>Então ele deve receber 1 curso gratuito adicional</t>
-  </si>
-  <si>
-    <t>E seu saldo de moedas deve ser debitado para 2 com a transferência gerada</t>
+    <t>Dado um aluno com assinatura básica ativa</t>
+  </si>
+  <si>
+    <t>com menos de 11 cursos concluídos</t>
+  </si>
+  <si>
+    <t>Quando o aluno conclui um curso</t>
+  </si>
+  <si>
+    <t>obtém nota final superior a 7,0</t>
+  </si>
+  <si>
+    <t>Então o sistema deve liberar o acesso a 3 novos cursos</t>
+  </si>
+  <si>
+    <t>manter a assinatura no plano básico</t>
+  </si>
+  <si>
+    <t>Dado um aluno com plano básico e 11 cursos concluídos</t>
+  </si>
+  <si>
+    <t>com todas as avaliações validadas</t>
+  </si>
+  <si>
+    <t>Quando o aluno conclui o seu 12º curso</t>
+  </si>
+  <si>
+    <t>Então a assinatura deve ser alterada para "Premium"</t>
+  </si>
+  <si>
+    <t>conceder 3 cursos, 3 moedas e voucher para projetos reais</t>
+  </si>
+  <si>
+    <t>matriculado em um curso da grade</t>
+  </si>
+  <si>
+    <t>Quando o aluno conclui o curso</t>
+  </si>
+  <si>
+    <t>obtém nota final igual ou inferior a 7,0</t>
+  </si>
+  <si>
+    <t>Então nenhum curso adicional deve ser liberado</t>
+  </si>
+  <si>
+    <t>o progresso para o plano Premium não deve ser incrementado</t>
   </si>
 </sst>
 </file>
@@ -760,7 +754,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -818,6 +812,21 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -860,19 +869,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -890,10 +887,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1095,104 +1088,104 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S1000"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" customWidth="1"/>
-    <col min="2" max="2" width="41.5546875" customWidth="1"/>
-    <col min="3" max="3" width="62.33203125" customWidth="1"/>
-    <col min="4" max="4" width="52.44140625" customWidth="1"/>
-    <col min="5" max="5" width="46.33203125" customWidth="1"/>
-    <col min="6" max="6" width="13.109375" customWidth="1"/>
-    <col min="7" max="7" width="53.44140625" customWidth="1"/>
-    <col min="8" max="8" width="47.6640625" customWidth="1"/>
-    <col min="9" max="9" width="60.44140625" customWidth="1"/>
-    <col min="10" max="10" width="50.5546875" customWidth="1"/>
-    <col min="11" max="11" width="57.6640625" customWidth="1"/>
-    <col min="12" max="12" width="46.44140625" customWidth="1"/>
-    <col min="13" max="13" width="8.44140625" customWidth="1"/>
+    <col min="1" max="1" width="7.28515625" customWidth="1"/>
+    <col min="2" max="2" width="41.5703125" customWidth="1"/>
+    <col min="3" max="3" width="62.28515625" customWidth="1"/>
+    <col min="4" max="4" width="52.42578125" customWidth="1"/>
+    <col min="5" max="5" width="46.28515625" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" customWidth="1"/>
+    <col min="7" max="7" width="53.42578125" customWidth="1"/>
+    <col min="8" max="8" width="47.7109375" customWidth="1"/>
+    <col min="9" max="9" width="60.42578125" customWidth="1"/>
+    <col min="10" max="10" width="50.5703125" customWidth="1"/>
+    <col min="11" max="11" width="57.7109375" customWidth="1"/>
+    <col min="12" max="12" width="46.42578125" customWidth="1"/>
+    <col min="13" max="13" width="8.42578125" customWidth="1"/>
     <col min="14" max="14" width="169" customWidth="1"/>
-    <col min="15" max="15" width="127.109375" customWidth="1"/>
-    <col min="16" max="16" width="36.5546875" customWidth="1"/>
+    <col min="15" max="15" width="127.140625" customWidth="1"/>
+    <col min="16" max="16" width="36.5703125" customWidth="1"/>
     <col min="17" max="17" width="39" customWidth="1"/>
-    <col min="18" max="18" width="8.44140625" customWidth="1"/>
-    <col min="19" max="19" width="46.33203125" customWidth="1"/>
-    <col min="20" max="26" width="8.44140625" customWidth="1"/>
+    <col min="18" max="18" width="8.42578125" customWidth="1"/>
+    <col min="19" max="19" width="46.28515625" customWidth="1"/>
+    <col min="20" max="26" width="8.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="55.5" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="27"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="32"/>
       <c r="F1" s="1"/>
-      <c r="G1" s="31" t="s">
+      <c r="G1" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="27"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="32"/>
       <c r="M1" s="1"/>
-      <c r="N1" s="32" t="s">
+      <c r="N1" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
-      <c r="Q1" s="26"/>
-      <c r="R1" s="26"/>
-      <c r="S1" s="27"/>
+      <c r="O1" s="31"/>
+      <c r="P1" s="31"/>
+      <c r="Q1" s="31"/>
+      <c r="R1" s="31"/>
+      <c r="S1" s="32"/>
     </row>
     <row r="2" spans="1:19" ht="26.25" customHeight="1">
-      <c r="A2" s="33"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
-      <c r="K2" s="34"/>
-      <c r="L2" s="34"/>
-      <c r="M2" s="34"/>
-      <c r="N2" s="34"/>
-      <c r="O2" s="34"/>
-      <c r="P2" s="34"/>
-      <c r="Q2" s="34"/>
-      <c r="R2" s="34"/>
-      <c r="S2" s="35"/>
+      <c r="A2" s="38"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
+      <c r="K2" s="39"/>
+      <c r="L2" s="39"/>
+      <c r="M2" s="39"/>
+      <c r="N2" s="39"/>
+      <c r="O2" s="39"/>
+      <c r="P2" s="39"/>
+      <c r="Q2" s="39"/>
+      <c r="R2" s="39"/>
+      <c r="S2" s="40"/>
     </row>
     <row r="3" spans="1:19" ht="36" customHeight="1">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="36" t="s">
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="26"/>
-      <c r="I3" s="26"/>
-      <c r="J3" s="26"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="27"/>
-      <c r="M3" s="40"/>
-      <c r="N3" s="36" t="s">
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="32"/>
+      <c r="M3" s="45"/>
+      <c r="N3" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="O3" s="26"/>
-      <c r="P3" s="26"/>
-      <c r="Q3" s="26"/>
-      <c r="R3" s="26"/>
-      <c r="S3" s="27"/>
+      <c r="O3" s="31"/>
+      <c r="P3" s="31"/>
+      <c r="Q3" s="31"/>
+      <c r="R3" s="31"/>
+      <c r="S3" s="32"/>
     </row>
     <row r="4" spans="1:19" ht="66" customHeight="1">
       <c r="A4" s="2" t="s">
@@ -1210,7 +1203,7 @@
       <c r="E4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="38"/>
+      <c r="F4" s="43"/>
       <c r="G4" s="3" t="s">
         <v>11</v>
       </c>
@@ -1229,37 +1222,37 @@
       <c r="L4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="M4" s="38"/>
+      <c r="M4" s="43"/>
       <c r="N4" s="3" t="s">
         <v>15</v>
       </c>
       <c r="O4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="P4" s="42" t="s">
+      <c r="P4" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="Q4" s="26"/>
-      <c r="R4" s="26"/>
-      <c r="S4" s="27"/>
+      <c r="Q4" s="31"/>
+      <c r="R4" s="31"/>
+      <c r="S4" s="32"/>
     </row>
     <row r="5" spans="1:19" ht="409.5" customHeight="1">
       <c r="A5" s="4">
         <v>1</v>
       </c>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="44" t="s">
+      <c r="D5" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="44" t="s">
+      <c r="E5" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="F5" s="38"/>
+      <c r="F5" s="43"/>
       <c r="G5" s="24" t="s">
         <v>46</v>
       </c>
@@ -1278,15 +1271,15 @@
       <c r="L5" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="M5" s="38"/>
+      <c r="M5" s="43"/>
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
-      <c r="P5" s="29"/>
-      <c r="Q5" s="26"/>
-      <c r="R5" s="26"/>
-      <c r="S5" s="27"/>
+      <c r="P5" s="34"/>
+      <c r="Q5" s="31"/>
+      <c r="R5" s="31"/>
+      <c r="S5" s="32"/>
     </row>
-    <row r="6" spans="1:19" ht="409.2" customHeight="1">
+    <row r="6" spans="1:19" ht="409.15" customHeight="1">
       <c r="A6" s="9"/>
       <c r="B6" s="20" t="s">
         <v>36</v>
@@ -1300,7 +1293,7 @@
       <c r="E6" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="F6" s="38"/>
+      <c r="F6" s="43"/>
       <c r="G6" s="24" t="s">
         <v>52</v>
       </c>
@@ -1311,62 +1304,62 @@
         <v>54</v>
       </c>
       <c r="J6" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="K6" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="K6" s="24" t="s">
+      <c r="L6" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="L6" s="24" t="s">
-        <v>57</v>
-      </c>
-      <c r="M6" s="38"/>
+      <c r="M6" s="43"/>
       <c r="N6" s="6"/>
       <c r="O6" s="6"/>
-      <c r="P6" s="29"/>
-      <c r="Q6" s="26"/>
-      <c r="R6" s="26"/>
-      <c r="S6" s="27"/>
+      <c r="P6" s="34"/>
+      <c r="Q6" s="31"/>
+      <c r="R6" s="31"/>
+      <c r="S6" s="32"/>
     </row>
     <row r="7" spans="1:19" ht="408.6" customHeight="1">
       <c r="A7" s="9"/>
-      <c r="B7" s="45" t="s">
+      <c r="B7" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="C7" s="46" t="s">
+      <c r="C7" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="47" t="s">
+      <c r="D7" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="47" t="s">
+      <c r="E7" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="F7" s="38"/>
+      <c r="F7" s="43"/>
       <c r="G7" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="H7" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="I7" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="H7" s="24" t="s">
+      <c r="J7" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="I7" s="24" t="s">
+      <c r="K7" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="J7" s="24" t="s">
+      <c r="L7" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="K7" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="L7" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="M7" s="38"/>
+      <c r="M7" s="43"/>
       <c r="N7" s="6"/>
       <c r="O7" s="5"/>
-      <c r="P7" s="25"/>
-      <c r="Q7" s="26"/>
-      <c r="R7" s="26"/>
-      <c r="S7" s="27"/>
+      <c r="P7" s="30"/>
+      <c r="Q7" s="31"/>
+      <c r="R7" s="31"/>
+      <c r="S7" s="32"/>
     </row>
     <row r="8" spans="1:19" ht="362.25" customHeight="1">
       <c r="A8" s="9"/>
@@ -1374,20 +1367,20 @@
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
-      <c r="F8" s="38"/>
+      <c r="F8" s="43"/>
       <c r="G8" s="6"/>
       <c r="H8" s="10"/>
       <c r="I8" s="6"/>
       <c r="J8" s="5"/>
-      <c r="K8" s="6"/>
+      <c r="K8" s="48"/>
       <c r="L8" s="10"/>
-      <c r="M8" s="38"/>
+      <c r="M8" s="43"/>
       <c r="N8" s="6"/>
       <c r="O8" s="5"/>
-      <c r="P8" s="28"/>
-      <c r="Q8" s="26"/>
-      <c r="R8" s="26"/>
-      <c r="S8" s="27"/>
+      <c r="P8" s="33"/>
+      <c r="Q8" s="31"/>
+      <c r="R8" s="31"/>
+      <c r="S8" s="32"/>
     </row>
     <row r="9" spans="1:19" ht="355.5" customHeight="1">
       <c r="A9" s="9"/>
@@ -1395,20 +1388,20 @@
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
       <c r="E9" s="8"/>
-      <c r="F9" s="38"/>
+      <c r="F9" s="43"/>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
       <c r="L9" s="10"/>
-      <c r="M9" s="38"/>
+      <c r="M9" s="43"/>
       <c r="N9" s="6"/>
       <c r="O9" s="6"/>
-      <c r="P9" s="29"/>
-      <c r="Q9" s="26"/>
-      <c r="R9" s="26"/>
-      <c r="S9" s="27"/>
+      <c r="P9" s="34"/>
+      <c r="Q9" s="31"/>
+      <c r="R9" s="31"/>
+      <c r="S9" s="32"/>
     </row>
     <row r="10" spans="1:19" ht="201" hidden="1" customHeight="1">
       <c r="A10" s="9"/>
@@ -1416,20 +1409,20 @@
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
       <c r="E10" s="9"/>
-      <c r="F10" s="39"/>
+      <c r="F10" s="44"/>
       <c r="G10" s="9"/>
       <c r="H10" s="9"/>
       <c r="I10" s="9"/>
       <c r="J10" s="9"/>
       <c r="K10" s="9"/>
       <c r="L10" s="9"/>
-      <c r="M10" s="39"/>
+      <c r="M10" s="44"/>
       <c r="N10" s="9"/>
       <c r="O10" s="9"/>
-      <c r="P10" s="41"/>
-      <c r="Q10" s="26"/>
-      <c r="R10" s="26"/>
-      <c r="S10" s="27"/>
+      <c r="P10" s="46"/>
+      <c r="Q10" s="31"/>
+      <c r="R10" s="31"/>
+      <c r="S10" s="32"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -2431,105 +2424,105 @@
     <mergeCell ref="P6:S6"/>
   </mergeCells>
   <pageMargins left="0.51180555555555496" right="0.51180555555555496" top="0.78749999999999998" bottom="0.78749999999999998" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="27" orientation="landscape"/>
+  <pageSetup paperSize="9" scale="27" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A1000"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="63.33203125" customWidth="1"/>
-    <col min="2" max="26" width="8.44140625" customWidth="1"/>
+    <col min="1" max="1" width="63.28515625" customWidth="1"/>
+    <col min="2" max="26" width="8.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="57.6">
+    <row r="1" spans="1:1" ht="60">
       <c r="A1" s="11" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="14.4">
+    <row r="2" spans="1:1">
       <c r="A2" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="28.8">
+    <row r="3" spans="1:1" ht="30">
       <c r="A3" s="12" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="14.4">
+    <row r="4" spans="1:1">
       <c r="A4" s="13"/>
     </row>
-    <row r="5" spans="1:1" ht="14.4">
+    <row r="5" spans="1:1">
       <c r="A5" s="12" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="14.4">
+    <row r="6" spans="1:1">
       <c r="A6" s="9"/>
     </row>
-    <row r="7" spans="1:1" ht="14.4">
+    <row r="7" spans="1:1">
       <c r="A7" s="14" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="14.4">
+    <row r="8" spans="1:1">
       <c r="A8" s="15" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="14.4">
+    <row r="9" spans="1:1">
       <c r="A9" s="16" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="14.4">
+    <row r="10" spans="1:1">
       <c r="A10" s="9"/>
     </row>
-    <row r="11" spans="1:1" ht="14.4">
+    <row r="11" spans="1:1">
       <c r="A11" s="9"/>
     </row>
-    <row r="12" spans="1:1" ht="14.4">
+    <row r="12" spans="1:1">
       <c r="A12" s="15" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="14.4">
+    <row r="13" spans="1:1">
       <c r="A13" s="17" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="14.4">
+    <row r="14" spans="1:1">
       <c r="A14" s="18" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="14.4">
+    <row r="15" spans="1:1">
       <c r="A15" s="17" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="14.4">
+    <row r="16" spans="1:1">
       <c r="A16" s="9"/>
     </row>
-    <row r="17" spans="1:1" ht="14.4">
+    <row r="17" spans="1:1">
       <c r="A17" s="15" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="14.4">
+    <row r="18" spans="1:1">
       <c r="A18" s="19" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="14.4">
+    <row r="19" spans="1:1">
       <c r="A19" s="18" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="14.4">
+    <row r="20" spans="1:1">
       <c r="A20" s="17" t="s">
         <v>32</v>
       </c>

</xml_diff>